<commit_message>
Updated IPL Auction system with login, bidding, logout
</commit_message>
<xml_diff>
--- a/players.xlsx
+++ b/players.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,6 +493,11 @@
           <t>last_bid_time</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>current Bid</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -517,7 +522,7 @@
         <v>20000000</v>
       </c>
       <c r="F2" t="n">
-        <v>400000000</v>
+        <v>9900000000</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -537,8 +542,9 @@
         <v>4</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>46087.49066140856</v>
-      </c>
+        <v>46087.50706166666</v>
+      </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -583,6 +589,7 @@
         <v>15</v>
       </c>
       <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -627,6 +634,7 @@
         <v>145</v>
       </c>
       <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -671,6 +679,7 @@
         <v>28</v>
       </c>
       <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -715,6 +724,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -759,6 +769,7 @@
         <v>53</v>
       </c>
       <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -803,6 +814,7 @@
         <v>0</v>
       </c>
       <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -847,6 +859,7 @@
         <v>139</v>
       </c>
       <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>